<commit_message>
Corrected Silicat Potasium into 2 different groups
</commit_message>
<xml_diff>
--- a/estimation_output/fertilizer_price_estimations_2025-08-13_12-47-51.xlsx
+++ b/estimation_output/fertilizer_price_estimations_2025-08-13_12-47-51.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\webscraping\estimation_output\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76E5F983-8EC7-4F74-AB3E-BC7C1E930E26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Fertilizer_Price_Estimations" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -973,8 +979,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1037,13 +1043,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1081,7 +1095,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1115,6 +1129,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1149,9 +1164,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1324,11 +1340,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H79"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1354,7 +1373,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1371,7 +1390,7 @@
         <v>1416666.666666667</v>
       </c>
       <c r="F2">
-        <v>312472.0905595581</v>
+        <v>312472.09055955813</v>
       </c>
       <c r="G2" t="s">
         <v>164</v>
@@ -1380,7 +1399,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1397,7 +1416,7 @@
         <v>1600000</v>
       </c>
       <c r="F3">
-        <v>450852.749866701</v>
+        <v>450852.74986670102</v>
       </c>
       <c r="G3" t="s">
         <v>165</v>
@@ -1406,7 +1425,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1414,7 +1433,7 @@
         <v>88</v>
       </c>
       <c r="C4">
-        <v>364270.8333333334</v>
+        <v>364270.83333333337</v>
       </c>
       <c r="D4">
         <v>2500</v>
@@ -1423,7 +1442,7 @@
         <v>1000000</v>
       </c>
       <c r="F4">
-        <v>278569.4574520101</v>
+        <v>278569.45745201007</v>
       </c>
       <c r="G4" t="s">
         <v>166</v>
@@ -1432,7 +1451,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -1455,7 +1474,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1478,7 +1497,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1501,7 +1520,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -1518,7 +1537,7 @@
         <v>980000</v>
       </c>
       <c r="F8">
-        <v>326339.2917399518</v>
+        <v>326339.29173995182</v>
       </c>
       <c r="G8" t="s">
         <v>170</v>
@@ -1527,7 +1546,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -1550,7 +1569,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1558,7 +1577,7 @@
         <v>94</v>
       </c>
       <c r="C10">
-        <v>620186.3354037267</v>
+        <v>620186.33540372667</v>
       </c>
       <c r="D10">
         <v>320000</v>
@@ -1567,7 +1586,7 @@
         <v>4890000</v>
       </c>
       <c r="F10">
-        <v>2189520.869796803</v>
+        <v>2189520.8697968032</v>
       </c>
       <c r="G10" t="s">
         <v>172</v>
@@ -1576,7 +1595,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -1599,7 +1618,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -1622,7 +1641,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -1645,7 +1664,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -1668,7 +1687,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -1691,7 +1710,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -1708,7 +1727,7 @@
         <v>420000</v>
       </c>
       <c r="F16">
-        <v>53033.00858899106</v>
+        <v>53033.008588991062</v>
       </c>
       <c r="G16" t="s">
         <v>178</v>
@@ -1717,7 +1736,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -1740,7 +1759,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>24</v>
       </c>
@@ -1757,7 +1776,7 @@
         <v>111000</v>
       </c>
       <c r="F18">
-        <v>39495.65201104772</v>
+        <v>39495.652011047721</v>
       </c>
       <c r="G18" t="s">
         <v>180</v>
@@ -1766,7 +1785,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -1792,7 +1811,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>26</v>
       </c>
@@ -1809,7 +1828,7 @@
         <v>700000</v>
       </c>
       <c r="F20">
-        <v>197907.5673346861</v>
+        <v>197907.56733468609</v>
       </c>
       <c r="G20" t="s">
         <v>182</v>
@@ -1818,7 +1837,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>27</v>
       </c>
@@ -1844,7 +1863,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>28</v>
       </c>
@@ -1861,7 +1880,7 @@
         <v>1300000</v>
       </c>
       <c r="F22">
-        <v>410374.0043354884</v>
+        <v>410374.00433548843</v>
       </c>
       <c r="G22" t="s">
         <v>184</v>
@@ -1870,7 +1889,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="23" spans="1:8">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>29</v>
       </c>
@@ -1896,7 +1915,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="24" spans="1:8">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>30</v>
       </c>
@@ -1913,7 +1932,7 @@
         <v>1330000</v>
       </c>
       <c r="F24">
-        <v>366678.405733036</v>
+        <v>366678.40573303599</v>
       </c>
       <c r="G24" t="s">
         <v>186</v>
@@ -1922,7 +1941,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>31</v>
       </c>
@@ -1945,7 +1964,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="26" spans="1:8">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>32</v>
       </c>
@@ -1971,7 +1990,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="27" spans="1:8">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>33</v>
       </c>
@@ -1988,7 +2007,7 @@
         <v>152000</v>
       </c>
       <c r="F27">
-        <v>57178.08437971085</v>
+        <v>57178.084379710846</v>
       </c>
       <c r="G27" t="s">
         <v>189</v>
@@ -1997,7 +2016,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>34</v>
       </c>
@@ -2014,7 +2033,7 @@
         <v>170000</v>
       </c>
       <c r="F28">
-        <v>108187.3375215418</v>
+        <v>108187.33752154181</v>
       </c>
       <c r="G28" t="s">
         <v>190</v>
@@ -2023,7 +2042,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>35</v>
       </c>
@@ -2049,7 +2068,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>36</v>
       </c>
@@ -2072,7 +2091,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>37</v>
       </c>
@@ -2080,16 +2099,16 @@
         <v>115</v>
       </c>
       <c r="C31">
-        <v>687291.6666666667</v>
+        <v>687291.66666666674</v>
       </c>
       <c r="D31">
-        <v>384583.3333333334</v>
+        <v>384583.33333333337</v>
       </c>
       <c r="E31">
         <v>990000</v>
       </c>
       <c r="F31">
-        <v>428094.2304433556</v>
+        <v>428094.23044335563</v>
       </c>
       <c r="G31" t="s">
         <v>193</v>
@@ -2098,7 +2117,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>38</v>
       </c>
@@ -2121,7 +2140,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>39</v>
       </c>
@@ -2138,7 +2157,7 @@
         <v>580000</v>
       </c>
       <c r="F33">
-        <v>138492.9011101101</v>
+        <v>138492.90111011011</v>
       </c>
       <c r="G33" t="s">
         <v>195</v>
@@ -2147,7 +2166,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>40</v>
       </c>
@@ -2164,7 +2183,7 @@
         <v>1550000</v>
       </c>
       <c r="F34">
-        <v>806101.7305526641</v>
+        <v>806101.73055266414</v>
       </c>
       <c r="G34" t="s">
         <v>196</v>
@@ -2173,7 +2192,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="35" spans="1:8">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>41</v>
       </c>
@@ -2190,7 +2209,7 @@
         <v>1116666.666666667</v>
       </c>
       <c r="F35">
-        <v>535568.4501674972</v>
+        <v>535568.45016749715</v>
       </c>
       <c r="G35" t="s">
         <v>197</v>
@@ -2199,7 +2218,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>42</v>
       </c>
@@ -2216,7 +2235,7 @@
         <v>930000</v>
       </c>
       <c r="F36">
-        <v>302567.0788386762</v>
+        <v>302567.07883867621</v>
       </c>
       <c r="G36" t="s">
         <v>198</v>
@@ -2225,7 +2244,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>43</v>
       </c>
@@ -2251,7 +2270,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>44</v>
       </c>
@@ -2268,7 +2287,7 @@
         <v>556000</v>
       </c>
       <c r="F38">
-        <v>46669.04755831214</v>
+        <v>46669.047558312137</v>
       </c>
       <c r="G38" t="s">
         <v>200</v>
@@ -2277,7 +2296,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>45</v>
       </c>
@@ -2294,7 +2313,7 @@
         <v>76000</v>
       </c>
       <c r="F39">
-        <v>52184.48045156721</v>
+        <v>52184.480451567208</v>
       </c>
       <c r="G39" t="s">
         <v>201</v>
@@ -2303,7 +2322,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="40" spans="1:8">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>46</v>
       </c>
@@ -2320,7 +2339,7 @@
         <v>300000</v>
       </c>
       <c r="F40">
-        <v>138524.3660877032</v>
+        <v>138524.36608770321</v>
       </c>
       <c r="G40" t="s">
         <v>202</v>
@@ -2329,7 +2348,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="41" spans="1:8">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>47</v>
       </c>
@@ -2346,7 +2365,7 @@
         <v>550000</v>
       </c>
       <c r="F41">
-        <v>158707.8632731074</v>
+        <v>158707.86327310739</v>
       </c>
       <c r="G41" t="s">
         <v>203</v>
@@ -2355,7 +2374,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="42" spans="1:8">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>48</v>
       </c>
@@ -2372,7 +2391,7 @@
         <v>134000</v>
       </c>
       <c r="F42">
-        <v>44046.82151658943</v>
+        <v>44046.821516589429</v>
       </c>
       <c r="G42" t="s">
         <v>204</v>
@@ -2381,7 +2400,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="43" spans="1:8">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>49</v>
       </c>
@@ -2398,7 +2417,7 @@
         <v>1840000</v>
       </c>
       <c r="F43">
-        <v>846834.7221664134</v>
+        <v>846834.72216641344</v>
       </c>
       <c r="G43" t="s">
         <v>205</v>
@@ -2407,7 +2426,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="44" spans="1:8">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>50</v>
       </c>
@@ -2418,13 +2437,13 @@
         <v>785000</v>
       </c>
       <c r="D44">
-        <v>253571.4285714286</v>
+        <v>253571.42857142861</v>
       </c>
       <c r="E44">
         <v>7500000</v>
       </c>
       <c r="F44">
-        <v>3105424.869876742</v>
+        <v>3105424.8698767419</v>
       </c>
       <c r="G44" t="s">
         <v>206</v>
@@ -2433,7 +2452,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="45" spans="1:8">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>51</v>
       </c>
@@ -2459,7 +2478,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="46" spans="1:8">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>52</v>
       </c>
@@ -2476,7 +2495,7 @@
         <v>920000</v>
       </c>
       <c r="F46">
-        <v>242898.6022034317</v>
+        <v>242898.60220343171</v>
       </c>
       <c r="G46" t="s">
         <v>208</v>
@@ -2485,7 +2504,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="47" spans="1:8">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>53</v>
       </c>
@@ -2493,7 +2512,7 @@
         <v>131</v>
       </c>
       <c r="C47">
-        <v>416666.6666666667</v>
+        <v>416666.66666666669</v>
       </c>
       <c r="D47">
         <v>139200</v>
@@ -2502,7 +2521,7 @@
         <v>650000</v>
       </c>
       <c r="F47">
-        <v>184934.7457397289</v>
+        <v>184934.74573972891</v>
       </c>
       <c r="G47" t="s">
         <v>209</v>
@@ -2511,7 +2530,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="48" spans="1:8">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>54</v>
       </c>
@@ -2528,7 +2547,7 @@
         <v>1083333.333333333</v>
       </c>
       <c r="F48">
-        <v>247563.5047596655</v>
+        <v>247563.50475966549</v>
       </c>
       <c r="G48" t="s">
         <v>210</v>
@@ -2537,7 +2556,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="49" spans="1:8">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>55</v>
       </c>
@@ -2554,7 +2573,7 @@
         <v>5926000</v>
       </c>
       <c r="F49">
-        <v>2233569.878020386</v>
+        <v>2233569.8780203862</v>
       </c>
       <c r="G49" t="s">
         <v>211</v>
@@ -2563,7 +2582,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="50" spans="1:8">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>56</v>
       </c>
@@ -2586,7 +2605,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="51" spans="1:8">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>57</v>
       </c>
@@ -2603,7 +2622,7 @@
         <v>850000</v>
       </c>
       <c r="F51">
-        <v>283058.5502279393</v>
+        <v>283058.55022793933</v>
       </c>
       <c r="G51" t="s">
         <v>213</v>
@@ -2612,7 +2631,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="52" spans="1:8">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>58</v>
       </c>
@@ -2626,7 +2645,7 @@
         <v>97000</v>
       </c>
       <c r="E52">
-        <v>323529.4117647058</v>
+        <v>323529.41176470579</v>
       </c>
       <c r="F52">
         <v>119205.0001176818</v>
@@ -2638,7 +2657,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="53" spans="1:8">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>59</v>
       </c>
@@ -2661,7 +2680,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="54" spans="1:8">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>60</v>
       </c>
@@ -2684,7 +2703,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="55" spans="1:8">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>61</v>
       </c>
@@ -2707,7 +2726,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="56" spans="1:8">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>62</v>
       </c>
@@ -2724,7 +2743,7 @@
         <v>158800</v>
       </c>
       <c r="F56">
-        <v>86429.33529768698</v>
+        <v>86429.335297686979</v>
       </c>
       <c r="G56" t="s">
         <v>216</v>
@@ -2733,7 +2752,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="57" spans="1:8">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>63</v>
       </c>
@@ -2750,7 +2769,7 @@
         <v>121800</v>
       </c>
       <c r="F57">
-        <v>29530.1038802417</v>
+        <v>29530.103880241699</v>
       </c>
       <c r="G57" t="s">
         <v>217</v>
@@ -2759,7 +2778,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="58" spans="1:8">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>64</v>
       </c>
@@ -2776,7 +2795,7 @@
         <v>152500</v>
       </c>
       <c r="F58">
-        <v>38464.40454064857</v>
+        <v>38464.404540648567</v>
       </c>
       <c r="G58" t="s">
         <v>218</v>
@@ -2785,7 +2804,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="59" spans="1:8">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>65</v>
       </c>
@@ -2802,7 +2821,7 @@
         <v>400000</v>
       </c>
       <c r="F59">
-        <v>110611.2265068551</v>
+        <v>110611.22650685511</v>
       </c>
       <c r="G59" t="s">
         <v>219</v>
@@ -2811,7 +2830,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="60" spans="1:8">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>66</v>
       </c>
@@ -2828,7 +2847,7 @@
         <v>1700000</v>
       </c>
       <c r="F60">
-        <v>359563.2452838208</v>
+        <v>359563.24528382078</v>
       </c>
       <c r="G60" t="s">
         <v>220</v>
@@ -2837,7 +2856,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="61" spans="1:8">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>67</v>
       </c>
@@ -2854,7 +2873,7 @@
         <v>1940000</v>
       </c>
       <c r="F61">
-        <v>412513.1844408206</v>
+        <v>412513.18444082059</v>
       </c>
       <c r="G61" t="s">
         <v>221</v>
@@ -2863,7 +2882,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="62" spans="1:8">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>68</v>
       </c>
@@ -2886,7 +2905,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="63" spans="1:8">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>69</v>
       </c>
@@ -2903,7 +2922,7 @@
         <v>269000</v>
       </c>
       <c r="F63">
-        <v>179746.5437776204</v>
+        <v>179746.54377762039</v>
       </c>
       <c r="G63" t="s">
         <v>223</v>
@@ -2912,7 +2931,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="64" spans="1:8">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>70</v>
       </c>
@@ -2935,7 +2954,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="65" spans="1:8">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>71</v>
       </c>
@@ -2961,7 +2980,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="66" spans="1:8">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>72</v>
       </c>
@@ -2984,7 +3003,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="67" spans="1:8">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>73</v>
       </c>
@@ -3010,7 +3029,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="68" spans="1:8">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>74</v>
       </c>
@@ -3027,7 +3046,7 @@
         <v>26000000</v>
       </c>
       <c r="F68">
-        <v>17701711.16022403</v>
+        <v>17701711.160224032</v>
       </c>
       <c r="G68" t="s">
         <v>228</v>
@@ -3036,7 +3055,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="69" spans="1:8">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>75</v>
       </c>
@@ -3062,7 +3081,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="70" spans="1:8">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>76</v>
       </c>
@@ -3079,7 +3098,7 @@
         <v>3000000</v>
       </c>
       <c r="F70">
-        <v>910434.1631552866</v>
+        <v>910434.16315528657</v>
       </c>
       <c r="G70" t="s">
         <v>230</v>
@@ -3088,7 +3107,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="71" spans="1:8">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>77</v>
       </c>
@@ -3096,7 +3115,7 @@
         <v>155</v>
       </c>
       <c r="C71">
-        <v>716666.6666666667</v>
+        <v>716666.66666666674</v>
       </c>
       <c r="D71">
         <v>20000</v>
@@ -3105,7 +3124,7 @@
         <v>2560000</v>
       </c>
       <c r="F71">
-        <v>533197.1327315068</v>
+        <v>533197.13273150683</v>
       </c>
       <c r="G71" t="s">
         <v>231</v>
@@ -3114,7 +3133,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="72" spans="1:8">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>78</v>
       </c>
@@ -3137,7 +3156,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="73" spans="1:8">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>79</v>
       </c>
@@ -3154,7 +3173,7 @@
         <v>1400000</v>
       </c>
       <c r="F73">
-        <v>505107.2493375376</v>
+        <v>505107.24933753762</v>
       </c>
       <c r="G73" t="s">
         <v>233</v>
@@ -3163,7 +3182,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="74" spans="1:8">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>80</v>
       </c>
@@ -3189,7 +3208,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="75" spans="1:8">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>81</v>
       </c>
@@ -3203,10 +3222,10 @@
         <v>660000</v>
       </c>
       <c r="E75">
-        <v>1714285.714285714</v>
+        <v>1714285.7142857141</v>
       </c>
       <c r="F75">
-        <v>528093.4518411972</v>
+        <v>528093.45184119721</v>
       </c>
       <c r="G75" t="s">
         <v>235</v>
@@ -3215,7 +3234,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="76" spans="1:8">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>82</v>
       </c>
@@ -3232,7 +3251,7 @@
         <v>900000</v>
       </c>
       <c r="F76">
-        <v>256569.4787695837</v>
+        <v>256569.47876958369</v>
       </c>
       <c r="G76" t="s">
         <v>236</v>
@@ -3241,7 +3260,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="77" spans="1:8">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>83</v>
       </c>
@@ -3258,7 +3277,7 @@
         <v>1333333.333333333</v>
       </c>
       <c r="F77">
-        <v>355099.3595403606</v>
+        <v>355099.35954036057</v>
       </c>
       <c r="G77" t="s">
         <v>237</v>
@@ -3267,7 +3286,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="78" spans="1:8">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>84</v>
       </c>
@@ -3278,13 +3297,13 @@
         <v>14000</v>
       </c>
       <c r="D78">
-        <v>488.2352941176471</v>
+        <v>488.23529411764707</v>
       </c>
       <c r="E78">
         <v>25000</v>
       </c>
       <c r="F78">
-        <v>8570.560847264735</v>
+        <v>8570.5608472647345</v>
       </c>
       <c r="G78" t="s">
         <v>238</v>
@@ -3293,7 +3312,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="79" spans="1:8">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>85</v>
       </c>

</xml_diff>